<commit_message>
Update Premedical 1 bank soal with color-detected answer keys
Cross-reference font color/highlight markup in the source docx files
(red font, cyan/yellow/green highlight on the correct option) to fill
in more Jawaban values that plain-text extraction had missed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/edu/soal-premedical/Bank Soal UB Premedical 1.xlsx
+++ b/edu/soal-premedical/Bank Soal UB Premedical 1.xlsx
@@ -446,7 +446,7 @@
     <col width="28" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="45" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
   </cols>
@@ -739,7 +739,11 @@
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -864,7 +868,11 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -958,7 +966,11 @@
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1048,7 +1060,11 @@
       </c>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1189,7 +1205,11 @@
       </c>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1228,7 +1248,11 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Serabut Asosiasi: menghubungkan area dalam satu hemisfer otak. Serabut Komisural: menghubungkan kedua hemisfer (contoh: korpus kalosum). Serabut Proyeksi: menghubungkan otak dengan struktur di bawahnya (medulla spinalis).</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Serabut Asosiasi: menghubungkan area dalam satu hemisfer otak. Serabut Komisural: menghubungkan kedua hemisfer (contoh: korpus kalosum). Serabut Proyeksi: menghubungkan otak dengan struktur di bawahnya (medulla spinalis).</t>
@@ -1795,7 +1819,11 @@
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2940,7 +2968,11 @@
           <t>Areolare</t>
         </is>
       </c>
-      <c r="M53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N53" s="2" t="inlineStr"/>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3066,7 +3098,11 @@
           <t>Makrofag</t>
         </is>
       </c>
-      <c r="M55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N55" s="2" t="inlineStr"/>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3129,7 +3165,11 @@
           <t>Peningkatan kalsium di sitosol</t>
         </is>
       </c>
-      <c r="M56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N56" s="2" t="inlineStr"/>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3192,7 +3232,11 @@
           <t>Serabut retikuler</t>
         </is>
       </c>
-      <c r="M57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N57" s="2" t="inlineStr"/>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3326,7 +3370,11 @@
           <t>Natrium</t>
         </is>
       </c>
-      <c r="M59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N59" s="2" t="inlineStr"/>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3389,7 +3437,11 @@
           <t>Katalase</t>
         </is>
       </c>
-      <c r="M60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N60" s="2" t="inlineStr"/>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3452,7 +3504,11 @@
           <t>Inervasi neuron motorik somatic</t>
         </is>
       </c>
-      <c r="M61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N61" s="2" t="inlineStr"/>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3515,7 +3571,11 @@
           <t>M. infraspinatus</t>
         </is>
       </c>
-      <c r="M62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
           <t>Catatan pada opsi b: M. teres minor berperan pada abduksi horizontal, bukan sebagai prime mover abduksi bahu pada gerakan jumping jack.</t>
@@ -3582,7 +3642,11 @@
           <t>Soma</t>
         </is>
       </c>
-      <c r="M63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N63" s="2" t="inlineStr"/>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3645,7 +3709,11 @@
           <t>Selenium</t>
         </is>
       </c>
-      <c r="M64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N64" s="2" t="inlineStr"/>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3708,7 +3776,11 @@
           <t>Kecepatan oksidasi asam lemak menjadi asetil KoA meningkat</t>
         </is>
       </c>
-      <c r="M65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N65" s="2" t="inlineStr"/>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3843,11 @@
           <t>Pediatric anatomy</t>
         </is>
       </c>
-      <c r="M66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N66" s="2" t="inlineStr"/>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3834,7 +3910,11 @@
           <t>Kreatin fosfat</t>
         </is>
       </c>
-      <c r="M67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N67" s="2" t="inlineStr"/>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -3897,7 +3977,11 @@
           <t>Peningkatan timbunan laktat dalam sel</t>
         </is>
       </c>
-      <c r="M68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N68" s="2" t="inlineStr"/>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -3960,7 +4044,11 @@
           <t>Sel hematopoetik</t>
         </is>
       </c>
-      <c r="M69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N69" s="2" t="inlineStr"/>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4023,7 +4111,11 @@
           <t>Kristalin</t>
         </is>
       </c>
-      <c r="M70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N70" s="2" t="inlineStr"/>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4086,7 +4178,11 @@
           <t>Lengan neuroglia lebih Panjang</t>
         </is>
       </c>
-      <c r="M71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N71" s="2" t="inlineStr"/>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4149,7 +4245,11 @@
           <t>Kanal natrium gerbang ligan</t>
         </is>
       </c>
-      <c r="M72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N72" s="2" t="inlineStr"/>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4212,7 +4312,11 @@
           <t>Kreatin fosfat dan AMP</t>
         </is>
       </c>
-      <c r="M73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N73" s="2" t="inlineStr"/>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4275,7 +4379,11 @@
           <t>Paru</t>
         </is>
       </c>
-      <c r="M74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N74" s="2" t="inlineStr"/>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4338,7 +4446,11 @@
           <t>Preacher hand</t>
         </is>
       </c>
-      <c r="M75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
           <t>Otot yang ditandai berwarna hijau pada gambar adalah M. Biceps Brachii. Ruptur tendon caput longum m. biceps brachii secara klasik memberikan gambaran Popeye sign.</t>
@@ -4405,7 +4517,11 @@
           <t>22</t>
         </is>
       </c>
-      <c r="M76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N76" s="2" t="inlineStr"/>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4468,7 +4584,11 @@
           <t>VL 1-2</t>
         </is>
       </c>
-      <c r="M77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
           <t>Sumber: MEDIAN EDISI 1 HAL.65</t>
@@ -4535,7 +4655,11 @@
           <t>Pembentukan vaskuler darah</t>
         </is>
       </c>
-      <c r="M78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N78" s="2" t="inlineStr"/>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4598,7 +4722,11 @@
           <t>Membuka kanal kalsium dan kalium</t>
         </is>
       </c>
-      <c r="M79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N79" s="2" t="inlineStr"/>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4661,7 +4789,11 @@
           <t>Superoksida dismutase</t>
         </is>
       </c>
-      <c r="M80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N80" s="2" t="inlineStr"/>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4724,7 +4856,11 @@
           <t>Pertumbuhan tulang hanya memanjang saja</t>
         </is>
       </c>
-      <c r="M81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
           <t>Catatan: pernyataan pada opsi a terbalik (seharusnya kondroblas berubah menjadi kondrosit); pernyataan pada opsi e juga kurang tepat karena pertumbuhan tulang tidak hanya memanjang tetapi juga menebal.</t>
@@ -4791,7 +4927,11 @@
           <t>2 ATP</t>
         </is>
       </c>
-      <c r="M82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N82" s="2" t="inlineStr"/>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4854,7 +4994,11 @@
           <t>Inspirasi tenang</t>
         </is>
       </c>
-      <c r="M83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N83" s="2" t="inlineStr"/>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4917,7 +5061,11 @@
           <t>Stimulasi fibroblast menjadi fibrosit</t>
         </is>
       </c>
-      <c r="M84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N84" s="2" t="inlineStr"/>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4980,7 +5128,11 @@
           <t>HPO₄²⁻</t>
         </is>
       </c>
-      <c r="M85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N85" s="2" t="inlineStr"/>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5195,11 @@
           <t>Cr</t>
         </is>
       </c>
-      <c r="M86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N86" s="2" t="inlineStr"/>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5106,7 +5262,11 @@
           <t>Power of hidrogen</t>
         </is>
       </c>
-      <c r="M87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N87" s="2" t="inlineStr"/>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5169,7 +5329,11 @@
           <t>Kelenjar adrenal</t>
         </is>
       </c>
-      <c r="M88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N88" s="2" t="inlineStr"/>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5555,7 +5719,11 @@
           <t>Melindungi otak dari infeksi bakteri</t>
         </is>
       </c>
-      <c r="M94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N94" s="2" t="inlineStr"/>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5618,7 +5786,11 @@
           <t>Interaksi penyelesaian konflik/masalah, frekuensi dan lamanya perdebatan, perilaku yang melekat selama konflik</t>
         </is>
       </c>
-      <c r="M95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N95" s="2" t="inlineStr"/>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5681,7 +5853,11 @@
           <t>3-fosfogliserat → 2 fosfogliserat</t>
         </is>
       </c>
-      <c r="M96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N96" s="2" t="inlineStr"/>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -6134,7 +6310,11 @@
           <t>Pengaturan mitogenic growth factor</t>
         </is>
       </c>
-      <c r="M103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N103" s="2" t="inlineStr"/>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -6197,7 +6377,11 @@
           <t>Fasciculus gracilis</t>
         </is>
       </c>
-      <c r="M104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N104" s="2" t="inlineStr"/>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6331,7 +6515,11 @@
           <t>Hati</t>
         </is>
       </c>
-      <c r="M106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N106" s="2" t="inlineStr"/>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6582,11 @@
           <t>Tersimpan tidak akan hilang</t>
         </is>
       </c>
-      <c r="M107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N107" s="2" t="inlineStr"/>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6528,7 +6720,11 @@
           <t>Madu</t>
         </is>
       </c>
-      <c r="M109" s="2" t="inlineStr"/>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N109" s="2" t="inlineStr"/>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6591,7 +6787,11 @@
           <t>Os. Maxilla</t>
         </is>
       </c>
-      <c r="M110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N110" s="2" t="inlineStr"/>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6654,7 +6854,11 @@
           <t>Oligodendrosit</t>
         </is>
       </c>
-      <c r="M111" s="2" t="inlineStr"/>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N111" s="2" t="inlineStr"/>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6717,7 +6921,11 @@
           <t>Myoblast</t>
         </is>
       </c>
-      <c r="M112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N112" s="2" t="inlineStr"/>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6922,7 +7130,11 @@
           <t>Reticulare astrocyte</t>
         </is>
       </c>
-      <c r="M115" s="2" t="inlineStr"/>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N115" s="2" t="inlineStr"/>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6985,7 +7197,11 @@
           <t>Ibu kandung</t>
         </is>
       </c>
-      <c r="M116" s="2" t="inlineStr"/>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N116" s="2" t="inlineStr"/>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -7048,7 +7264,11 @@
           <t>Interosea synchondrosis</t>
         </is>
       </c>
-      <c r="M117" s="2" t="inlineStr"/>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N117" s="2" t="inlineStr"/>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -7111,7 +7331,11 @@
           <t>Muskarinik</t>
         </is>
       </c>
-      <c r="M118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N118" s="2" t="inlineStr"/>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -7174,7 +7398,11 @@
           <t>Sistem saraf</t>
         </is>
       </c>
-      <c r="M119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N119" s="2" t="inlineStr"/>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -7379,7 +7607,11 @@
           <t>Fibroblast</t>
         </is>
       </c>
-      <c r="M122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N122" s="2" t="inlineStr"/>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -7442,7 +7674,11 @@
           <t>Growth hormone dan IGF-1</t>
         </is>
       </c>
-      <c r="M123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N123" s="2" t="inlineStr"/>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7505,7 +7741,11 @@
           <t>Information element</t>
         </is>
       </c>
-      <c r="M124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N124" s="2" t="inlineStr"/>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7568,7 +7808,11 @@
           <t>Fumarate menjadi malat</t>
         </is>
       </c>
-      <c r="M125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N125" s="2" t="inlineStr"/>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7631,7 +7875,11 @@
           <t>N. vagus</t>
         </is>
       </c>
-      <c r="M126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N126" s="2" t="inlineStr"/>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7694,7 +7942,11 @@
           <t>Biasa tidur miring</t>
         </is>
       </c>
-      <c r="M127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N127" s="2" t="inlineStr"/>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7757,7 +8009,11 @@
           <t>Fleksi-ekstensi</t>
         </is>
       </c>
-      <c r="M128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N128" s="2" t="inlineStr"/>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7820,7 +8076,11 @@
           <t>Galaktosa</t>
         </is>
       </c>
-      <c r="M129" s="2" t="inlineStr"/>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N129" s="2" t="inlineStr"/>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7883,7 +8143,11 @@
           <t>Nucleus sel otot jantung</t>
         </is>
       </c>
-      <c r="M130" s="2" t="inlineStr"/>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N130" s="2" t="inlineStr"/>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -8017,7 +8281,11 @@
           <t>Mengaktifkan second messenger untuk mengaktifkan ATP</t>
         </is>
       </c>
-      <c r="M132" s="2" t="inlineStr"/>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N132" s="2" t="inlineStr"/>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8411,11 @@
           <t>α-ketoglutarat dehidrogenase</t>
         </is>
       </c>
-      <c r="M134" s="2" t="inlineStr"/>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N134" s="2" t="inlineStr"/>
       <c r="O134" s="2" t="inlineStr">
         <is>
@@ -8206,7 +8478,11 @@
           <t>Articulatio humerodistalis</t>
         </is>
       </c>
-      <c r="M135" s="2" t="inlineStr"/>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N135" s="2" t="inlineStr"/>
       <c r="O135" s="2" t="inlineStr">
         <is>
@@ -8269,7 +8545,11 @@
           <t>Calbindin-D</t>
         </is>
       </c>
-      <c r="M136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N136" s="2" t="inlineStr"/>
       <c r="O136" s="2" t="inlineStr">
         <is>
@@ -8332,7 +8612,11 @@
           <t>Diet tinggi protein, pada metabolism normal menghasilkan lebih banyak basa daripada asam</t>
         </is>
       </c>
-      <c r="M137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N137" s="2" t="inlineStr"/>
       <c r="O137" s="2" t="inlineStr">
         <is>
@@ -8395,7 +8679,11 @@
           <t>Vasodilatasi A. coronaria</t>
         </is>
       </c>
-      <c r="M138" s="2" t="inlineStr"/>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N138" s="2" t="inlineStr"/>
       <c r="O138" s="2" t="inlineStr">
         <is>
@@ -8458,7 +8746,11 @@
           <t>Reseptor</t>
         </is>
       </c>
-      <c r="M139" s="2" t="inlineStr"/>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N139" s="2" t="inlineStr"/>
       <c r="O139" s="2" t="inlineStr">
         <is>
@@ -8592,7 +8884,11 @@
           <t>M. gastrocnemius medialis, M. gastrocnemius lateralis, dan M. soleus</t>
         </is>
       </c>
-      <c r="M141" s="2" t="inlineStr"/>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N141" s="2" t="inlineStr"/>
       <c r="O141" s="2" t="inlineStr">
         <is>
@@ -8655,7 +8951,11 @@
           <t>Pyelonephritis</t>
         </is>
       </c>
-      <c r="M142" s="2" t="inlineStr"/>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N142" s="2" t="inlineStr"/>
       <c r="O142" s="2" t="inlineStr">
         <is>
@@ -8718,7 +9018,11 @@
           <t>Motor unit pekerja B lebih besar, namun ATP minimal</t>
         </is>
       </c>
-      <c r="M143" s="2" t="inlineStr"/>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N143" s="2" t="inlineStr"/>
       <c r="O143" s="2" t="inlineStr">
         <is>
@@ -8848,7 +9152,11 @@
           <t>Para simpatik</t>
         </is>
       </c>
-      <c r="M145" s="2" t="inlineStr"/>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N145" s="2" t="inlineStr"/>
       <c r="O145" s="2" t="inlineStr">
         <is>
@@ -8911,7 +9219,11 @@
           <t>Stasiun pemancar semua masukan sinaps</t>
         </is>
       </c>
-      <c r="M146" s="2" t="inlineStr"/>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N146" s="2" t="inlineStr"/>
       <c r="O146" s="2" t="inlineStr">
         <is>
@@ -8974,7 +9286,11 @@
           <t>Mengatur suhu tubuh</t>
         </is>
       </c>
-      <c r="M147" s="2" t="inlineStr"/>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N147" s="2" t="inlineStr"/>
       <c r="O147" s="2" t="inlineStr">
         <is>
@@ -9037,7 +9353,11 @@
           <t>Nilai ΔG positif</t>
         </is>
       </c>
-      <c r="M148" s="2" t="inlineStr"/>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N148" s="2" t="inlineStr"/>
       <c r="O148" s="2" t="inlineStr">
         <is>
@@ -9100,7 +9420,11 @@
           <t>1 pasang</t>
         </is>
       </c>
-      <c r="M149" s="2" t="inlineStr"/>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N149" s="2" t="inlineStr"/>
       <c r="O149" s="2" t="inlineStr">
         <is>
@@ -9163,7 +9487,11 @@
           <t>Pons</t>
         </is>
       </c>
-      <c r="M150" s="2" t="inlineStr"/>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N150" s="2" t="inlineStr"/>
       <c r="O150" s="2" t="inlineStr">
         <is>
@@ -9226,7 +9554,11 @@
           <t>One</t>
         </is>
       </c>
-      <c r="M151" s="2" t="inlineStr"/>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N151" s="2" t="inlineStr"/>
       <c r="O151" s="2" t="inlineStr">
         <is>
@@ -9289,7 +9621,11 @@
           <t>Hematoxylin eosin</t>
         </is>
       </c>
-      <c r="M152" s="2" t="inlineStr"/>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N152" s="2" t="inlineStr"/>
       <c r="O152" s="2" t="inlineStr">
         <is>
@@ -9809,7 +10145,11 @@
           <t>Pembentukan asam laktat</t>
         </is>
       </c>
-      <c r="M160" s="2" t="inlineStr"/>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N160" s="2" t="inlineStr"/>
       <c r="O160" s="2" t="inlineStr">
         <is>
@@ -9872,7 +10212,11 @@
           <t>Proses yang tidak memerlukan coupling dengan reaksi lain</t>
         </is>
       </c>
-      <c r="M161" s="2" t="inlineStr"/>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N161" s="2" t="inlineStr"/>
       <c r="O161" s="2" t="inlineStr">
         <is>
@@ -9935,7 +10279,11 @@
           <t>Sel fibroblast</t>
         </is>
       </c>
-      <c r="M162" s="2" t="inlineStr"/>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N162" s="2" t="inlineStr"/>
       <c r="O162" s="2" t="inlineStr">
         <is>
@@ -9998,7 +10346,11 @@
           <t>Kuboid simplek</t>
         </is>
       </c>
-      <c r="M163" s="2" t="inlineStr"/>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N163" s="2" t="inlineStr"/>
       <c r="O163" s="2" t="inlineStr">
         <is>
@@ -10057,7 +10409,11 @@
           <t>Potensial dalam serat saraf 90 mV lebih positif daripada potensial di cairan ekstrasel</t>
         </is>
       </c>
-      <c r="M164" s="2" t="inlineStr"/>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N164" s="2" t="inlineStr"/>
       <c r="O164" s="2" t="inlineStr">
         <is>
@@ -10120,7 +10476,11 @@
           <t>Menyediakan sisa metabolism sel dan medium reaksi kimia</t>
         </is>
       </c>
-      <c r="M165" s="2" t="inlineStr"/>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N165" s="2" t="inlineStr"/>
       <c r="O165" s="2" t="inlineStr">
         <is>
@@ -10459,7 +10819,11 @@
           <t>Na+</t>
         </is>
       </c>
-      <c r="M170" s="2" t="inlineStr"/>
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N170" s="2" t="inlineStr"/>
       <c r="O170" s="2" t="inlineStr">
         <is>
@@ -10522,7 +10886,11 @@
           <t>Kreatin fosfat dan AMP</t>
         </is>
       </c>
-      <c r="M171" s="2" t="inlineStr"/>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N171" s="2" t="inlineStr"/>
       <c r="O171" s="2" t="inlineStr">
         <is>
@@ -10585,7 +10953,11 @@
           <t>Tembaga</t>
         </is>
       </c>
-      <c r="M172" s="2" t="inlineStr"/>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N172" s="2" t="inlineStr"/>
       <c r="O172" s="2" t="inlineStr">
         <is>
@@ -10719,7 +11091,11 @@
           <t>Osmosis</t>
         </is>
       </c>
-      <c r="M174" s="2" t="inlineStr"/>
+      <c r="M174" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N174" s="2" t="inlineStr"/>
       <c r="O174" s="2" t="inlineStr">
         <is>
@@ -10782,7 +11158,11 @@
           <t>Komunikasi jarak jauh (potensial aksi)</t>
         </is>
       </c>
-      <c r="M175" s="2" t="inlineStr"/>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N175" s="2" t="inlineStr">
         <is>
           <t>Aktivasi saluran ion gated menyebabkan potensial aksi pada potensial bertingkat.</t>
@@ -10849,7 +11229,11 @@
           <t>N. trigeminus</t>
         </is>
       </c>
-      <c r="M176" s="2" t="inlineStr"/>
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N176" s="2" t="inlineStr"/>
       <c r="O176" s="2" t="inlineStr">
         <is>
@@ -11113,7 +11497,11 @@
         </is>
       </c>
       <c r="L180" s="2" t="inlineStr"/>
-      <c r="M180" s="2" t="inlineStr"/>
+      <c r="M180" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N180" s="2" t="inlineStr"/>
       <c r="O180" s="2" t="inlineStr">
         <is>
@@ -11176,7 +11564,11 @@
           <t>Mampu melakukan regenerasi terbatas</t>
         </is>
       </c>
-      <c r="M181" s="2" t="inlineStr"/>
+      <c r="M181" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N181" s="2" t="inlineStr"/>
       <c r="O181" s="2" t="inlineStr">
         <is>
@@ -11239,7 +11631,11 @@
           <t>Columna cranii</t>
         </is>
       </c>
-      <c r="M182" s="2" t="inlineStr"/>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N182" s="2" t="inlineStr"/>
       <c r="O182" s="2" t="inlineStr">
         <is>
@@ -11304,7 +11700,7 @@
       </c>
       <c r="M183" s="2" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>E</t>
         </is>
       </c>
       <c r="N183" s="2" t="inlineStr">
@@ -11373,7 +11769,11 @@
           <t>M. Masseter</t>
         </is>
       </c>
-      <c r="M184" s="2" t="inlineStr"/>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N184" s="2" t="inlineStr"/>
       <c r="O184" s="2" t="inlineStr">
         <is>
@@ -11436,7 +11836,11 @@
           <t>Pada proses-proses yang spontan, entropi cenderung menurun</t>
         </is>
       </c>
-      <c r="M185" s="2" t="inlineStr"/>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N185" s="2" t="inlineStr"/>
       <c r="O185" s="2" t="inlineStr">
         <is>
@@ -11499,7 +11903,11 @@
           <t>Power stroke</t>
         </is>
       </c>
-      <c r="M186" s="2" t="inlineStr"/>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N186" s="2" t="inlineStr"/>
       <c r="O186" s="2" t="inlineStr">
         <is>
@@ -11562,7 +11970,11 @@
           <t>Bradikardi</t>
         </is>
       </c>
-      <c r="M187" s="2" t="inlineStr"/>
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N187" s="2" t="inlineStr"/>
       <c r="O187" s="2" t="inlineStr">
         <is>
@@ -11625,7 +12037,11 @@
           <t>Bersamaan dengan makan lemak</t>
         </is>
       </c>
-      <c r="M188" s="2" t="inlineStr"/>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N188" s="2" t="inlineStr"/>
       <c r="O188" s="2" t="inlineStr">
         <is>
@@ -11684,7 +12100,11 @@
         </is>
       </c>
       <c r="L189" s="2" t="inlineStr"/>
-      <c r="M189" s="2" t="inlineStr"/>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N189" s="2" t="inlineStr">
         <is>
           <t>Catatan pada sumber teks: "kalium adalah kofaktor mineral" - namun tidak ada opsi kalium sehingga catatan ini kemungkinan keliru/tidak sesuai pilihan yang tersedia.</t>
@@ -11751,7 +12171,11 @@
           <t>Lapisan multiformis</t>
         </is>
       </c>
-      <c r="M190" s="2" t="inlineStr"/>
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N190" s="2" t="inlineStr"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
@@ -11814,7 +12238,11 @@
           <t>Mempertahankan arsitektur tulang</t>
         </is>
       </c>
-      <c r="M191" s="2" t="inlineStr"/>
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N191" s="2" t="inlineStr"/>
       <c r="O191" s="2" t="inlineStr">
         <is>
@@ -11877,7 +12305,11 @@
           <t>Baroreseptor dan osmoreseptor</t>
         </is>
       </c>
-      <c r="M192" s="2" t="inlineStr"/>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N192" s="2" t="inlineStr"/>
       <c r="O192" s="2" t="inlineStr">
         <is>
@@ -11940,7 +12372,11 @@
           <t>Memodulasi pelepasan katekolamin</t>
         </is>
       </c>
-      <c r="M193" s="2" t="inlineStr"/>
+      <c r="M193" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N193" s="2" t="inlineStr"/>
       <c r="O193" s="2" t="inlineStr">
         <is>
@@ -12070,7 +12506,11 @@
           <t>Ganglion radix posterior</t>
         </is>
       </c>
-      <c r="M195" s="2" t="inlineStr"/>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N195" s="2" t="inlineStr"/>
       <c r="O195" s="2" t="inlineStr">
         <is>
@@ -12133,7 +12573,11 @@
           <t>Fossa olecranon dengan olecranon</t>
         </is>
       </c>
-      <c r="M196" s="2" t="inlineStr"/>
+      <c r="M196" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N196" s="2" t="inlineStr"/>
       <c r="O196" s="2" t="inlineStr">
         <is>
@@ -12198,7 +12642,7 @@
       </c>
       <c r="M197" s="2" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>A</t>
         </is>
       </c>
       <c r="N197" s="2" t="inlineStr">
@@ -12330,7 +12774,11 @@
           <t>Rangsangan - peningkatan ion Ca intra sel - Ion Ca berikatan dengan troponin - Pengaktifan kinase - Fosforilasi aktin - Miosin berikatan dengan aktin</t>
         </is>
       </c>
-      <c r="M199" s="2" t="inlineStr"/>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N199" s="2" t="inlineStr"/>
       <c r="O199" s="2" t="inlineStr">
         <is>
@@ -12393,7 +12841,11 @@
           <t>Inervasi motorik otonom</t>
         </is>
       </c>
-      <c r="M200" s="2" t="inlineStr"/>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N200" s="2" t="inlineStr"/>
       <c r="O200" s="2" t="inlineStr">
         <is>
@@ -12456,7 +12908,11 @@
           <t>Fossa acetabuli</t>
         </is>
       </c>
-      <c r="M201" s="2" t="inlineStr"/>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N201" s="2" t="inlineStr"/>
       <c r="O201" s="2" t="inlineStr">
         <is>
@@ -12519,7 +12975,11 @@
           <t>Representasi bagian wajah lebih lebar daripada kaki</t>
         </is>
       </c>
-      <c r="M202" s="2" t="inlineStr"/>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N202" s="2" t="inlineStr"/>
       <c r="O202" s="2" t="inlineStr">
         <is>
@@ -12582,7 +13042,11 @@
           <t>Kompleks I</t>
         </is>
       </c>
-      <c r="M203" s="2" t="inlineStr"/>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N203" s="2" t="inlineStr"/>
       <c r="O203" s="2" t="inlineStr">
         <is>
@@ -12645,7 +13109,11 @@
           <t>Kapasitas tidak terbatas</t>
         </is>
       </c>
-      <c r="M204" s="2" t="inlineStr"/>
+      <c r="M204" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N204" s="2" t="inlineStr"/>
       <c r="O204" s="2" t="inlineStr">
         <is>
@@ -12708,7 +13176,11 @@
           <t>Peningkatan CO2 darah</t>
         </is>
       </c>
-      <c r="M205" s="2" t="inlineStr"/>
+      <c r="M205" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N205" s="2" t="inlineStr"/>
       <c r="O205" s="2" t="inlineStr">
         <is>
@@ -12773,7 +13245,7 @@
       </c>
       <c r="M206" s="2" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>C</t>
         </is>
       </c>
       <c r="N206" s="2" t="inlineStr">
@@ -12842,7 +13314,11 @@
           <t>Xanthin oksidase</t>
         </is>
       </c>
-      <c r="M207" s="2" t="inlineStr"/>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N207" s="2" t="inlineStr"/>
       <c r="O207" s="2" t="inlineStr">
         <is>
@@ -12905,7 +13381,11 @@
           <t>Intestinum tenue and colon proksimal</t>
         </is>
       </c>
-      <c r="M208" s="2" t="inlineStr"/>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N208" s="2" t="inlineStr"/>
       <c r="O208" s="2" t="inlineStr">
         <is>
@@ -13039,7 +13519,11 @@
           <t>Eritrosit mulai menggunakan benda keton sebagai sumber energinya</t>
         </is>
       </c>
-      <c r="M210" s="2" t="inlineStr"/>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N210" s="2" t="inlineStr"/>
       <c r="O210" s="2" t="inlineStr">
         <is>
@@ -13102,7 +13586,11 @@
           <t>Serat kolagen membentuk berkas padat</t>
         </is>
       </c>
-      <c r="M211" s="2" t="inlineStr"/>
+      <c r="M211" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N211" s="2" t="inlineStr"/>
       <c r="O211" s="2" t="inlineStr">
         <is>
@@ -13165,7 +13653,11 @@
           <t>Osteosit</t>
         </is>
       </c>
-      <c r="M212" s="2" t="inlineStr"/>
+      <c r="M212" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N212" s="2" t="inlineStr"/>
       <c r="O212" s="2" t="inlineStr">
         <is>
@@ -13228,7 +13720,11 @@
           <t>Kanal K tertutup dan kanal Na masih tertutup</t>
         </is>
       </c>
-      <c r="M213" s="2" t="inlineStr"/>
+      <c r="M213" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N213" s="2" t="inlineStr"/>
       <c r="O213" s="2" t="inlineStr">
         <is>
@@ -13291,7 +13787,11 @@
           <t>Difusi terfasilitasi yang diperantarai carrier</t>
         </is>
       </c>
-      <c r="M214" s="2" t="inlineStr"/>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N214" s="2" t="inlineStr"/>
       <c r="O214" s="2" t="inlineStr">
         <is>
@@ -13417,7 +13917,11 @@
           <t>Tempat replikasi DNA</t>
         </is>
       </c>
-      <c r="M216" s="2" t="inlineStr"/>
+      <c r="M216" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N216" s="2" t="inlineStr"/>
       <c r="O216" s="2" t="inlineStr">
         <is>
@@ -13480,7 +13984,11 @@
           <t>Aspartat</t>
         </is>
       </c>
-      <c r="M217" s="2" t="inlineStr"/>
+      <c r="M217" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N217" s="2" t="inlineStr"/>
       <c r="O217" s="2" t="inlineStr">
         <is>
@@ -13606,7 +14114,11 @@
           <t>Kartilago Elastis</t>
         </is>
       </c>
-      <c r="M219" s="2" t="inlineStr"/>
+      <c r="M219" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N219" s="2" t="inlineStr"/>
       <c r="O219" s="2" t="inlineStr">
         <is>
@@ -13669,7 +14181,11 @@
           <t>m. Teres minor</t>
         </is>
       </c>
-      <c r="M220" s="2" t="inlineStr"/>
+      <c r="M220" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="N220" s="2" t="inlineStr"/>
       <c r="O220" s="2" t="inlineStr">
         <is>
@@ -13732,7 +14248,11 @@
           <t>Gap junction</t>
         </is>
       </c>
-      <c r="M221" s="2" t="inlineStr"/>
+      <c r="M221" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N221" s="2" t="inlineStr"/>
       <c r="O221" s="2" t="inlineStr">
         <is>
@@ -13921,7 +14441,11 @@
           <t>38 ATP</t>
         </is>
       </c>
-      <c r="M224" s="2" t="inlineStr"/>
+      <c r="M224" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N224" s="2" t="inlineStr"/>
       <c r="O224" s="2" t="inlineStr">
         <is>
@@ -14173,7 +14697,11 @@
           <t>Asam piruvat</t>
         </is>
       </c>
-      <c r="M228" s="2" t="inlineStr"/>
+      <c r="M228" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N228" s="2" t="inlineStr"/>
       <c r="O228" s="2" t="inlineStr">
         <is>
@@ -15016,7 +15544,11 @@
           <t>Calsium influx</t>
         </is>
       </c>
-      <c r="M241" s="2" t="inlineStr"/>
+      <c r="M241" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N241" s="2" t="inlineStr"/>
       <c r="O241" s="2" t="inlineStr">
         <is>
@@ -15205,7 +15737,11 @@
           <t>Inhibitor kompleks 2 rantai respirasi</t>
         </is>
       </c>
-      <c r="M244" s="2" t="inlineStr"/>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N244" s="2" t="inlineStr"/>
       <c r="O244" s="2" t="inlineStr">
         <is>
@@ -15268,7 +15804,11 @@
           <t>Bersifat avaskuler</t>
         </is>
       </c>
-      <c r="M245" s="2" t="inlineStr"/>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N245" s="2" t="inlineStr"/>
       <c r="O245" s="2" t="inlineStr">
         <is>
@@ -15394,7 +15934,11 @@
           <t>Rotasi-sirkumduksi</t>
         </is>
       </c>
-      <c r="M247" s="2" t="inlineStr"/>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="N247" s="2" t="inlineStr"/>
       <c r="O247" s="2" t="inlineStr">
         <is>
@@ -15457,7 +16001,11 @@
           <t>-94 mV</t>
         </is>
       </c>
-      <c r="M248" s="2" t="inlineStr"/>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="N248" s="2" t="inlineStr"/>
       <c r="O248" s="2" t="inlineStr">
         <is>
@@ -15520,7 +16068,11 @@
           <t>Membrana basalis</t>
         </is>
       </c>
-      <c r="M249" s="2" t="inlineStr"/>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N249" s="2" t="inlineStr"/>
       <c r="O249" s="2" t="inlineStr">
         <is>
@@ -15583,7 +16135,11 @@
           <t>Fasciculus arcuatus</t>
         </is>
       </c>
-      <c r="M250" s="2" t="inlineStr"/>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N250" s="2" t="inlineStr"/>
       <c r="O250" s="2" t="inlineStr">
         <is>
@@ -15646,7 +16202,11 @@
           <t>Disebut juga tulang hasta</t>
         </is>
       </c>
-      <c r="M251" s="2" t="inlineStr"/>
+      <c r="M251" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N251" s="2" t="inlineStr"/>
       <c r="O251" s="2" t="inlineStr">
         <is>
@@ -15709,7 +16269,11 @@
           <t>Berukuran lebih besar dibanding neuroglia</t>
         </is>
       </c>
-      <c r="M252" s="2" t="inlineStr"/>
+      <c r="M252" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
       <c r="N252" s="2" t="inlineStr"/>
       <c r="O252" s="2" t="inlineStr">
         <is>
@@ -15772,7 +16336,11 @@
           <t>Peningkatan filtrasi kapiler</t>
         </is>
       </c>
-      <c r="M253" s="2" t="inlineStr"/>
+      <c r="M253" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N253" s="2" t="inlineStr"/>
       <c r="O253" s="2" t="inlineStr">
         <is>
@@ -15965,7 +16533,11 @@
           <t>Lordosis thoracalis</t>
         </is>
       </c>
-      <c r="M256" s="2" t="inlineStr"/>
+      <c r="M256" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="N256" s="2" t="inlineStr"/>
       <c r="O256" s="2" t="inlineStr">
         <is>

</xml_diff>